<commit_message>
Tracker: record the audit's six QA results and three security findings
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documents/BACKLOG_Tracker.xlsx
+++ b/Documents/BACKLOG_Tracker.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blockers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E01 Blockers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Results" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Plan" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Backlog" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Blockers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="E01 Blockers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="QA Results" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Security Findings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sprint Plan" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Reference" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog'!$A$4:$W$197</definedName>
@@ -468,7 +468,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -629,6 +629,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1313,13 +1316,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1342,7 +1345,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1373,13 +1376,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1403,7 +1406,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1427,7 +1430,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1456,8 +1459,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1483,8 +1486,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1510,13 +1513,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1540,7 +1543,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1568,8 +1571,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1604,13 +1607,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1629,7 +1632,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1672,8 +1675,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1696,13 +1699,13 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1725,7 +1728,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1756,13 +1759,13 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1786,7 +1789,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1829,8 +1832,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1853,7 +1856,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -1868,9 +1871,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1890,9 +1893,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1912,9 +1915,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1934,9 +1937,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1946,7 +1949,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>8</col>
@@ -1961,9 +1964,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1973,7 +1976,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -1988,9 +1991,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21056,7 +21059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="59" min="1" max="1"/>
@@ -22599,17 +22602,17 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="65" t="inlineStr">
+      <c r="A44" s="67" t="inlineStr">
         <is>
           <t>QA-E02-09</t>
         </is>
       </c>
-      <c r="B44" s="65" t="inlineStr">
+      <c r="B44" s="67" t="inlineStr">
         <is>
           <t>E02-S04</t>
         </is>
       </c>
-      <c r="C44" s="65" t="inlineStr">
+      <c r="C44" s="67" t="inlineStr">
         <is>
           <t>BA: acceptance criteria re-checked against code</t>
         </is>
@@ -22634,6 +22637,246 @@
           <t>test_broker_security.py</t>
         </is>
       </c>
+    </row>
+    <row r="45" ht="86" customHeight="1" s="59">
+      <c r="A45" s="67" t="inlineStr">
+        <is>
+          <t>QA-AUD-01</t>
+        </is>
+      </c>
+      <c r="B45" s="67" t="inlineStr">
+        <is>
+          <t>E05/E06</t>
+        </is>
+      </c>
+      <c r="C45" s="67" t="inlineStr">
+        <is>
+          <t>Architecture: does anything compose the components?</t>
+        </is>
+      </c>
+      <c r="D45" s="66" t="inlineStr">
+        <is>
+          <t>FAIL (on plan)</t>
+        </is>
+      </c>
+      <c r="E45" s="67" t="inlineStr">
+        <is>
+          <t>Measured, not read: six service packages (orchestrator, signals, execution, premarket, api, notifier) are 1 line each - __init__.py only. No module in src/ imports both algotrader.ingest and algotrader.indicators. Zero production callers for set_atr_pct, set_circuit, MultiTimeframeBuilder, CleaningPipeline, QuotePublisher or warm_up_symbols.</t>
+        </is>
+      </c>
+      <c r="F45" s="67" t="inlineStr">
+        <is>
+          <t>~7,000 lines of tested components with no assembly. Expected at this point - E07 is the orchestrator - but it means no test so far is an end-to-end test of the SYSTEM. Recorded so the gap is explicit rather than assumed.</t>
+        </is>
+      </c>
+      <c r="G45" s="67" t="inlineStr">
+        <is>
+          <t>grep over src/</t>
+        </is>
+      </c>
+      <c r="H45" s="76" t="n"/>
+      <c r="I45" s="76" t="n"/>
+      <c r="J45" s="76" t="n"/>
+    </row>
+    <row r="46" ht="86" customHeight="1" s="59">
+      <c r="A46" s="67" t="inlineStr">
+        <is>
+          <t>QA-AUD-02</t>
+        </is>
+      </c>
+      <c r="B46" s="67" t="inlineStr">
+        <is>
+          <t>E05/E06</t>
+        </is>
+      </c>
+      <c r="C46" s="67" t="inlineStr">
+        <is>
+          <t>Architecture: the ingest/indicator dependency cycle</t>
+        </is>
+      </c>
+      <c r="D46" s="66" t="inlineStr">
+        <is>
+          <t>PASS (documented)</t>
+        </is>
+      </c>
+      <c r="E46" s="67" t="inlineStr">
+        <is>
+          <t>OutlierFilter needs ATR (E06) &lt;- needs bars (E05) &lt;- needs cleaned ticks &lt;- needs OutlierFilter. Reads as an unbreakable runtime loop.</t>
+        </is>
+      </c>
+      <c r="F46" s="67" t="inlineStr">
+        <is>
+          <t>It is not a loop: the ATR that matters is the PREVIOUS session's, loaded from ohlcv at warm-up before the feed connects. The hazard is the wiring, not the design - feeding it live bars would widen the threshold in response to the very outliers it rejects, each bad print raising ATR and each raised ATR admitting a worse one. Now stated in CleaningPipeline's docstring where the wiring will be written.</t>
+        </is>
+      </c>
+      <c r="G46" s="67" t="inlineStr">
+        <is>
+          <t>cleaning.py CleaningPipeline docstring</t>
+        </is>
+      </c>
+      <c r="H46" s="76" t="n"/>
+      <c r="I46" s="76" t="n"/>
+      <c r="J46" s="76" t="n"/>
+    </row>
+    <row r="47" ht="86" customHeight="1" s="59">
+      <c r="A47" s="67" t="inlineStr">
+        <is>
+          <t>QA-AUD-03</t>
+        </is>
+      </c>
+      <c r="B47" s="67" t="inlineStr">
+        <is>
+          <t>E06-S01</t>
+        </is>
+      </c>
+      <c r="C47" s="67" t="inlineStr">
+        <is>
+          <t>BA: performance criterion measured, not assumed</t>
+        </is>
+      </c>
+      <c r="D47" s="66" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E47" s="67" t="inlineStr">
+        <is>
+          <t>Budget is 50ms for a full indicator update cycle. Measured 3.9ms for 1200 indicator sets - 12x under budget.</t>
+        </is>
+      </c>
+      <c r="F47" s="67" t="inlineStr">
+        <is>
+          <t>The criterion was written as a target and had never been measured against real volume.</t>
+        </is>
+      </c>
+      <c r="G47" s="67" t="inlineStr">
+        <is>
+          <t>audit probe, 1200 sets</t>
+        </is>
+      </c>
+      <c r="H47" s="76" t="n"/>
+      <c r="I47" s="76" t="n"/>
+      <c r="J47" s="76" t="n"/>
+    </row>
+    <row r="48" ht="86" customHeight="1" s="59">
+      <c r="A48" s="67" t="inlineStr">
+        <is>
+          <t>QA-AUD-04</t>
+        </is>
+      </c>
+      <c r="B48" s="67" t="inlineStr">
+        <is>
+          <t>E05-S06</t>
+        </is>
+      </c>
+      <c r="C48" s="67" t="inlineStr">
+        <is>
+          <t>BA: full-session bar grid verified end to end</t>
+        </is>
+      </c>
+      <c r="D48" s="66" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E48" s="67" t="inlineStr">
+        <is>
+          <t>A complete 09:15-15:30 session produced 74 five-minute bars with 0 off-grid boundaries.</t>
+        </is>
+      </c>
+      <c r="F48" s="67" t="inlineStr">
+        <is>
+          <t>Bars align to the session start, not wall-clock hours. An off-by-one here shifts every indicator value for the day.</t>
+        </is>
+      </c>
+      <c r="G48" s="67" t="inlineStr">
+        <is>
+          <t>audit probe, full session replay</t>
+        </is>
+      </c>
+      <c r="H48" s="76" t="n"/>
+      <c r="I48" s="76" t="n"/>
+      <c r="J48" s="76" t="n"/>
+    </row>
+    <row r="49" ht="86" customHeight="1" s="59">
+      <c r="A49" s="67" t="inlineStr">
+        <is>
+          <t>QA-AUD-05</t>
+        </is>
+      </c>
+      <c r="B49" s="67" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="C49" s="67" t="inlineStr">
+        <is>
+          <t>BA: acceptance criteria not met</t>
+        </is>
+      </c>
+      <c r="D49" s="66" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E49" s="67" t="inlineStr">
+        <is>
+          <t>Two gaps: (1) FeedGap is produced by KiteFeed and IndicatorSet.mark_stale exists, but nothing connects them - a feed gap does not currently mark indicators stale because no component owns both. (2) ADX is named in the story and is not implemented.</t>
+        </is>
+      </c>
+      <c r="F49" s="67" t="inlineStr">
+        <is>
+          <t>Both are consequences of QA-AUD-01 rather than defects in the built code. (1) closes when the orchestrator lands; (2) is a straightforward addition to the indicator framework.</t>
+        </is>
+      </c>
+      <c r="G49" s="67" t="inlineStr">
+        <is>
+          <t>acceptance criteria re-read against code</t>
+        </is>
+      </c>
+      <c r="H49" s="76" t="n"/>
+      <c r="I49" s="76" t="n"/>
+      <c r="J49" s="76" t="n"/>
+    </row>
+    <row r="50" ht="86" customHeight="1" s="59">
+      <c r="A50" s="67" t="inlineStr">
+        <is>
+          <t>QA-AUD-06</t>
+        </is>
+      </c>
+      <c r="B50" s="67" t="inlineStr">
+        <is>
+          <t>E05/E06</t>
+        </is>
+      </c>
+      <c r="C50" s="67" t="inlineStr">
+        <is>
+          <t>Money-path type discipline</t>
+        </is>
+      </c>
+      <c r="D50" s="66" t="inlineStr">
+        <is>
+          <t>FAIL -&gt; Fixed</t>
+        </is>
+      </c>
+      <c r="E50" s="67" t="inlineStr">
+        <is>
+          <t>ATR.value returns float 1.4000000000000057 and ATR feeds stop distance, which feeds position size. CLAUDE.md requires Decimal for all money.</t>
+        </is>
+      </c>
+      <c r="F50" s="67" t="inlineStr">
+        <is>
+          <t>Indicators compute in float deliberately - they are the numerical-library boundary the conventions carve out, and TA-Lib parity is defined in float. So the fix is a NAMED crossing (as_decimal()) rather than scattered Decimal() calls at whichever site needs one. .value stays float for the indicator path.</t>
+        </is>
+      </c>
+      <c r="G50" s="67" t="inlineStr">
+        <is>
+          <t>test_indicators.py TestTheMoneyBoundaryIsExplicit</t>
+        </is>
+      </c>
+      <c r="H50" s="76" t="n"/>
+      <c r="I50" s="76" t="n"/>
+      <c r="J50" s="76" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:G20"/>
@@ -22652,7 +22895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="59" min="1" max="1"/>
@@ -23396,17 +23639,17 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="65" t="inlineStr">
+      <c r="A20" s="67" t="inlineStr">
         <is>
           <t>QA-SEC-16</t>
         </is>
       </c>
-      <c r="B20" s="65" t="inlineStr">
+      <c r="B20" s="67" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C20" s="65" t="inlineStr">
+      <c r="C20" s="67" t="inlineStr">
         <is>
           <t>Order logging / symbol handling</t>
         </is>
@@ -23437,6 +23680,141 @@
           <t>6 hostile symbols refused (newline, CRLF, colon, glob, over-length, empty) plus a CONTROL that real Indian symbols still work: M&amp;M, BAJAJ-AUTO, L&amp;TFH, NIFTY.NS, IDEA_EQ</t>
         </is>
       </c>
+    </row>
+    <row r="21" ht="92" customHeight="1" s="59">
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t>QA-SEC-17</t>
+        </is>
+      </c>
+      <c r="B21" s="67" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C21" s="67" t="inlineStr">
+        <is>
+          <t>Indicator state restore (E06)</t>
+        </is>
+      </c>
+      <c r="D21" s="66" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E21" s="67" t="inlineStr">
+        <is>
+          <t>restore() accepted period: -5 from a snapshot. EMA alpha became -0.5 - an indicator that DIVERGES instead of converging while emitting plausible numbers the whole time. Observed: a restored EMA drifting away from price with no error, no exception, no log line.</t>
+        </is>
+      </c>
+      <c r="F21" s="67" t="inlineStr">
+        <is>
+          <t>__init__ validated its period; restore() did not, and restore() is the path that reads state which has round-tripped through Redis. A partially-written key or a version skew between processes is enough - no attacker required. Nothing downstream can detect a wrong-but-plausible indicator value, so this fails OPEN, which the invariants forbid.</t>
+        </is>
+      </c>
+      <c r="G21" s="67" t="inlineStr">
+        <is>
+          <t>_checked_period() applied at all 8 restore sites (SMA, EMA, RSI, ATR, Bollinger, VolumeRatio, Wilder, MACD fast+slow). A corrupt period now raises IndicatorError rather than constructing a diverging indicator.</t>
+        </is>
+      </c>
+      <c r="H21" s="67" t="inlineStr">
+        <is>
+          <t>9 parametrised cases across 6 indicator types (negative, zero, non-numeric, None) plus a CONTROL that a valid snapshot still restores identically to a re-warmed set</t>
+        </is>
+      </c>
+      <c r="I21" s="76" t="n"/>
+      <c r="J21" s="76" t="n"/>
+      <c r="K21" s="76" t="n"/>
+    </row>
+    <row r="22" ht="92" customHeight="1" s="59">
+      <c r="A22" s="67" t="inlineStr">
+        <is>
+          <t>QA-SEC-18</t>
+        </is>
+      </c>
+      <c r="B22" s="67" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C22" s="67" t="inlineStr">
+        <is>
+          <t>Tick deduplication (E05)</t>
+        </is>
+      </c>
+      <c r="D22" s="66" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E22" s="67" t="inlineStr">
+        <is>
+          <t>The per-instrument dedup window was bounded at 512; the map holding those windows was not. 5000 distinct tokens produced 5000 retained windows with nothing to evict them.</t>
+        </is>
+      </c>
+      <c r="F22" s="67" t="inlineStr">
+        <is>
+          <t>Memory growth for the life of the process on a feed that churns instrument tokens - re-listings, corporate actions, a subscription list that changes daily. Not remotely triggerable, but it is an availability defect in a component meant to run a full session unattended.</t>
+        </is>
+      </c>
+      <c r="G22" s="67" t="inlineStr">
+        <is>
+          <t>The instrument map is now an LRU bounded at 1024. A universe of 200 fits several times over, so eviction only ever reaches symbols that genuinely stopped ticking.</t>
+        </is>
+      </c>
+      <c r="H22" s="67" t="inlineStr">
+        <is>
+          <t>3 tests: the map stays bounded across 1000 tokens; a continuously-ticking symbol survives 200 others churning past it; the original per-instrument bound still holds</t>
+        </is>
+      </c>
+      <c r="I22" s="76" t="n"/>
+      <c r="J22" s="76" t="n"/>
+      <c r="K22" s="76" t="n"/>
+    </row>
+    <row r="23" ht="92" customHeight="1" s="59">
+      <c r="A23" s="67" t="inlineStr">
+        <is>
+          <t>QA-SEC-19</t>
+        </is>
+      </c>
+      <c r="B23" s="67" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C23" s="67" t="inlineStr">
+        <is>
+          <t>Rate-limit error handling</t>
+        </is>
+      </c>
+      <c r="D23" s="66" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E23" s="67" t="inlineStr">
+        <is>
+          <t>Two exception classes were both named RateLimitError with OPPOSITE retry semantics. broker.adapter.RateLimitError means back off and retry; redis.primitives.RateLimitError meant the bucket is misconfigured and will never allow anything through.</t>
+        </is>
+      </c>
+      <c r="F23" s="67" t="inlineStr">
+        <is>
+          <t>A caller importing either name and wrapping it in the standard retry-with-backoff gets correct behaviour for one and an INFINITE LOOP for the other - against a condition that never clears. No test would fail, because the misconfigured bucket never becomes healthy and the loop never exits. In a component that gates order submission, a hang is a fail-open.</t>
+        </is>
+      </c>
+      <c r="G23" s="67" t="inlineStr">
+        <is>
+          <t>Renamed the Redis one to RateLimiterConfigError, with a docstring stating why the two are named apart.</t>
+        </is>
+      </c>
+      <c r="H23" s="67" t="inlineStr">
+        <is>
+          <t>3 tests: the types are distinct, neither is a subclass of the other, and only the broker one is reported by is_retryable()</t>
+        </is>
+      </c>
+      <c r="I23" s="76" t="n"/>
+      <c r="J23" s="76" t="n"/>
+      <c r="K23" s="76" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:H11"/>

</xml_diff>

<commit_message>
Tracker: record the SIT round for E14-S03
QA-E14-17. Twelve SIT scenarios, no product defect found. The one test that
failed on its first run was the test: it filtered a session walk on
`reason is RISK_ENGINE_FAULT` and swept up every clean minute, because with no
sizer configured a fully-cleared candidate is refused by the sizer under that
same reason. Session.stopped_by() reads the audit `stage` instead.

Recorded rather than quietly fixed, because filtering a session by reason code
is a natural thing to write and is quietly wrong the moment more than one
condition maps to one reason -- which SIT-001's fix deliberately arranged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documents/BACKLOG_Tracker.xlsx
+++ b/Documents/BACKLOG_Tracker.xlsx
@@ -4572,7 +4572,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="59">
       <c r="A4" s="37" t="inlineStr">
         <is>
@@ -21323,7 +21322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="59" min="1" max="1"/>
@@ -24267,6 +24266,43 @@
       <c r="G79" s="76" t="inlineStr">
         <is>
           <t>full suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="76" t="inlineStr">
+        <is>
+          <t>QA-E14-17</t>
+        </is>
+      </c>
+      <c r="B80" s="76" t="inlineStr">
+        <is>
+          <t>E14-S03</t>
+        </is>
+      </c>
+      <c r="C80" s="76" t="inlineStr">
+        <is>
+          <t>SIT: eligibility walked across a session</t>
+        </is>
+      </c>
+      <c r="D80" s="76" t="inlineStr">
+        <is>
+          <t>PASS (no product defect)</t>
+        </is>
+      </c>
+      <c r="E80" s="76" t="inlineStr">
+        <is>
+          <t>12 scenarios: the composition property (all seven clear on exactly the minutes four did -- 340 either way), a symbol banned at noon, an eligibility fetcher dropping out for 30 minutes and returning, the book filling and freeing, a position opened mid-session that correctly never releases, ordering across both check groups at every minute, audit completeness with seven registered, QA-SEC-30 at session scale, and replay determinism. SIT total 31 -&gt; 43.</t>
+        </is>
+      </c>
+      <c r="F80" s="76" t="inlineStr">
+        <is>
+          <t>One test failed on the first run and it was the TEST, not the product: it filtered the session on `reason is RISK_ENGINE_FAULT` and swept up every clean minute, because with no sizer configured a fully-cleared candidate is refused BY THE SIZER carrying that same reason. Added Session.stopped_by(), which reads the audit `stage` -- the field that actually answers 'which check refused'. Recorded because filtering a session by reason code is a natural thing to write and quietly wrong once more than one condition maps to a reason. No SIT defect logged.</t>
+        </is>
+      </c>
+      <c r="G80" s="76" t="inlineStr">
+        <is>
+          <t>tests/sit/test_e14_trading_session.py TestSit6 (12 tests)</t>
         </is>
       </c>
     </row>
@@ -24316,7 +24352,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
         <is>

</xml_diff>